<commit_message>
Externalize resistance databases and add DB metadata to reports
</commit_message>
<xml_diff>
--- a/data/db/cmv/resistances.xlsx
+++ b/data/db/cmv/resistances.xlsx
@@ -5,10 +5,11 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="resistances" sheetId="1" state="visible" r:id="rId2"/>
+    <sheet name="metadata" sheetId="2" state="visible" r:id="rId3"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -20,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="18">
   <si>
     <t xml:space="preserve">CHROM</t>
   </si>
@@ -63,6 +64,18 @@
   <si>
     <t xml:space="preserve">NA</t>
   </si>
+  <si>
+    <t xml:space="preserve">key</t>
+  </si>
+  <si>
+    <t xml:space="preserve">value</t>
+  </si>
+  <si>
+    <t xml:space="preserve">db_name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">no database</t>
+  </si>
 </sst>
 </file>
 
@@ -72,7 +85,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="&quot;VERDADERO&quot;;&quot;VERDADERO&quot;;&quot;FALSO&quot;"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -111,6 +124,13 @@
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
@@ -164,7 +184,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -199,6 +219,14 @@
     </xf>
     <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -3480,4 +3508,47 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData>
+    <row r="1" customFormat="false" ht="13.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="35.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="B2" s="10" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="9"/>
+      <c r="B3" s="9"/>
+    </row>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="10"/>
+      <c r="B4" s="10"/>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Normal"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Normal"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>